<commit_message>
Abcdefu als generierter Song, Tabelle mit Spalten Effekt / Änderungswunsch
- Abcdefu (#15): generierte Fassung ersetzt den Aufruf in main.cpp, alter Code
  bleibt in songs.cpp. Alte Effekte 1:1 übernommen, dazu: Pause ganz schwarz,
  Texte "A B C D E" vor jedem Chorus und "FUCK YOU" auf den Chorus-Einsatz
  (Chorus 1 schwarz ausgestanzt), "FUCK OFF" über dem Strobo, Blinder am Stopp,
  SCENE_VERSE nach dem Stopp, Schluss-Strobo im Viertel-Raster.
- Tabelle: der User trägt Wünsche in "Änderungswunsch" ein, songgen.py schreibt
  bei jeder Generierung den umgesetzten Effekt in "Effekt (füllt KI)"
  (struktur.write_effects mit Kontrolle nach dem Schreiben, neues Kommando
  --tabelle, alte Tabellen mit "Effektidee" werden umgestellt, Vorlage angepasst).
- progText: ein Unterstrich wird als Leerzeichen gezeichnet, trennt aber nicht.
- Doku: CLAUDE.md, Skill new-song, Song-Workflow, README, FX-Pipeline-Plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/struktur-vorlage.xlsx
+++ b/songs/struktur-vorlage.xlsx
@@ -441,14 +441,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,7 +463,7 @@
           <t>Künstler</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>von takt = Taktnummer, an der der Part beginnt (ab 0 oder Taktnummern aus dem DAW). Halbe Takte als Kommazahl: 13,5.</t>
         </is>
@@ -477,7 +478,8 @@
       <c r="C2" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Erste Zeile = Pause am Anfang (schwarz). StartBit: so weit hinter ihrem Anfang kommt das Start-MIDI (0,125 = 1/8 · 0,25 = 1/4 · 0,375 = 3/8 Takt).</t>
         </is>
@@ -492,9 +494,10 @@
       <c r="C3" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Letzte Zeile 'Ende' = Schlusstakt des Songs; in ihrer Effektidee steht die Länge des Schluss-Blacks (z. B. 10 sek.).</t>
+      <c r="D3" s="3" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Letzte Zeile 'Ende' = Schlusstakt des Songs; in ihrer Spalte Effekt (oder Änderungswunsch) steht die Länge des Schluss-Blacks (z. B. 10 sek.).</t>
         </is>
       </c>
     </row>
@@ -507,9 +510,10 @@
       <c r="C4" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Effektidee = dein Wunsch für den Part (freier Text), Energie 0-5. BPM pro Part nur bei Tempowechsel überschreiben.</t>
+      <c r="D4" s="3" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Änderungswunsch = dein Wunsch für den Part (freier Text); erledigte Wünsche löschst du selbst. Effekt (füllt KI) = was gerade umgesetzt ist - schreibt das Skript bei jeder Generierung, dort nichts eintragen. Energie 0-5. BPM pro Part nur bei Tempowechsel überschreiben.</t>
         </is>
       </c>
     </row>
@@ -526,20 +530,25 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Effektidee</t>
+          <t>Effekt (füllt KI)</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
+          <t>Änderungswunsch</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>Energie 0-5</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>BPM pro Part</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Weitere Spalten (z. B. Beschreibung, Akkorde) sind erlaubt. Gleiche Partnamen werden automatisch nummeriert: chorus 1, chorus 1 (2) ...</t>
         </is>
@@ -554,15 +563,16 @@
           <t>pause</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>black</t>
         </is>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="E6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="6">
+      <c r="F6" s="6">
         <f>$C$3</f>
         <v/>
       </c>
@@ -576,15 +586,16 @@
           <t>intro</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>ruhig</t>
         </is>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="E7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="6">
+      <c r="F7" s="6">
         <f>$C$3</f>
         <v/>
       </c>
@@ -599,10 +610,11 @@
         </is>
       </c>
       <c r="C8" s="7" t="n"/>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="6">
+      <c r="F8" s="6">
         <f>$C$3</f>
         <v/>
       </c>
@@ -616,15 +628,16 @@
           <t>übergang</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>strobo</t>
         </is>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="E9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="6">
+      <c r="F9" s="6">
         <f>$C$3</f>
         <v/>
       </c>
@@ -638,15 +651,16 @@
           <t>chorus 1</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>action</t>
         </is>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="E10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="E10" s="6">
+      <c r="F10" s="6">
         <f>$C$3</f>
         <v/>
       </c>
@@ -665,10 +679,10 @@
           <t>10 sek. BLACK</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <f>$C$3</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Struktur-Tabelle: gerasterte Kopie (--raster) und gerasterte Vorlage
songgen.py <Song> --raster legt quelle/struktur-raster.xlsx an: dieselbe
Tabelle mit einer Zeile je Vierteltakt zwischen den Parts, je Part als
Excel-Gliederung eingeklappt. Die Tabelle des Users wird nur gelesen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/struktur-vorlage.xlsx
+++ b/songs/struktur-vorlage.xlsx
@@ -438,10 +438,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -478,7 +478,6 @@
       <c r="C2" s="3" t="n">
         <v>99</v>
       </c>
-      <c r="D2" s="3" t="n"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Erste Zeile = Pause am Anfang (schwarz). StartBit: so weit hinter ihrem Anfang kommt das Start-MIDI (0,125 = 1/8 · 0,25 = 1/4 · 0,375 = 3/8 Takt).</t>
@@ -494,7 +493,6 @@
       <c r="C3" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="D3" s="3" t="n"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Letzte Zeile 'Ende' = Schlusstakt des Songs; in ihrer Spalte Effekt (oder Änderungswunsch) steht die Länge des Schluss-Blacks (z. B. 10 sek.).</t>
@@ -510,10 +508,9 @@
       <c r="C4" s="3" t="n">
         <v>0.375</v>
       </c>
-      <c r="D4" s="3" t="n"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Änderungswunsch = dein Wunsch für den Part (freier Text); erledigte Wünsche löschst du selbst. Effekt (füllt KI) = was gerade umgesetzt ist - schreibt das Skript bei jeder Generierung, dort nichts eintragen. Energie 0-5. BPM pro Part nur bei Tempowechsel überschreiben.</t>
+          <t>Änderungswunsch = dein Wunsch für den Part (freier Text); erledigte Wünsche löschst du selbst. Effekt (füllt KI) = was gerade umgesetzt ist - schreibt das Skript bei jeder Generierung, dort nichts eintragen. Energie 0-5. BPM pro Part nur bei Abweichung vom BPM oben eintragen (leer = BPM oben).</t>
         </is>
       </c>
     </row>
@@ -554,7 +551,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" collapsed="1">
       <c r="A6" s="5" t="n">
         <v>0</v>
       </c>
@@ -572,119 +569,918 @@
       <c r="E6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="6">
-        <f>$C$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
+      <c r="F6" s="6" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Zwischenzeilen (von takt ohne Songpart) = eine Zeile je Vierteltakt, eingeklappt: Plus am linken Rand öffnet einen Part, der Knopf 2 oben links alle. Leer = der Effekt des Parts läuft weiter. Ein Änderungswunsch dort gilt genau für diese Stelle. Ein Songpart-Name dort macht daraus einen neuen Part.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" hidden="1" outlineLevel="1">
       <c r="A7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>intro</t>
-        </is>
-      </c>
+        <v>0.25</v>
+      </c>
+      <c r="B7" s="6" t="n"/>
       <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>ruhig</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="6">
-        <f>$C$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="H7" s="2" t="n"/>
+    </row>
+    <row r="8" hidden="1" outlineLevel="1">
       <c r="A8" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>verse 1</t>
-        </is>
-      </c>
+        <v>0.5</v>
+      </c>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="n"/>
-      <c r="E8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" s="6">
-        <f>$C$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="H8" s="2" t="n"/>
+    </row>
+    <row r="9" hidden="1" outlineLevel="1">
       <c r="A9" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>übergang</t>
-        </is>
-      </c>
+        <v>0.75</v>
+      </c>
+      <c r="B9" s="6" t="n"/>
       <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>strobo</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="6">
-        <f>$C$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="H9" s="2" t="n"/>
+    </row>
+    <row r="10" collapsed="1">
       <c r="A10" s="5" t="n">
-        <v>13.5</v>
+        <v>1</v>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>chorus 1</t>
+          <t>intro</t>
         </is>
       </c>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="inlineStr">
         <is>
+          <t>ruhig</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="6" t="n"/>
+    </row>
+    <row r="11" hidden="1" outlineLevel="1">
+      <c r="A11" s="5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+    </row>
+    <row r="12" hidden="1" outlineLevel="1">
+      <c r="A12" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+    </row>
+    <row r="13" hidden="1" outlineLevel="1">
+      <c r="A13" s="5" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+    </row>
+    <row r="14" hidden="1" outlineLevel="1">
+      <c r="A14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+    </row>
+    <row r="15" hidden="1" outlineLevel="1">
+      <c r="A15" s="5" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+    </row>
+    <row r="16" hidden="1" outlineLevel="1">
+      <c r="A16" s="5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+    </row>
+    <row r="17" hidden="1" outlineLevel="1">
+      <c r="A17" s="5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="7" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+    </row>
+    <row r="18" hidden="1" outlineLevel="1">
+      <c r="A18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+    </row>
+    <row r="19" hidden="1" outlineLevel="1">
+      <c r="A19" s="5" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+    </row>
+    <row r="20" hidden="1" outlineLevel="1">
+      <c r="A20" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+    </row>
+    <row r="21" hidden="1" outlineLevel="1">
+      <c r="A21" s="5" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+    </row>
+    <row r="22" hidden="1" outlineLevel="1">
+      <c r="A22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+    </row>
+    <row r="23" hidden="1" outlineLevel="1">
+      <c r="A23" s="5" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+    </row>
+    <row r="24" hidden="1" outlineLevel="1">
+      <c r="A24" s="5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1">
+      <c r="A25" s="5" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
+    <row r="26" collapsed="1">
+      <c r="A26" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>verse 1</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="6" t="n"/>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1">
+      <c r="A27" s="5" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+    </row>
+    <row r="28" hidden="1" outlineLevel="1">
+      <c r="A28" s="5" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1">
+      <c r="A29" s="5" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1">
+      <c r="A30" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1">
+      <c r="A31" s="5" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1">
+      <c r="A32" s="5" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1">
+      <c r="A33" s="5" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1">
+      <c r="A34" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1">
+      <c r="A35" s="5" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1">
+      <c r="A36" s="5" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1">
+      <c r="A37" s="5" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="7" t="n"/>
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="6" t="n"/>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1">
+      <c r="A38" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="n"/>
+    </row>
+    <row r="39" hidden="1" outlineLevel="1">
+      <c r="A39" s="5" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="n"/>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1">
+      <c r="A40" s="5" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1">
+      <c r="A41" s="5" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1">
+      <c r="A42" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1">
+      <c r="A43" s="5" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1">
+      <c r="A44" s="5" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="B44" s="6" t="n"/>
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="7" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1">
+      <c r="A45" s="5" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="7" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1">
+      <c r="A46" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="7" t="n"/>
+      <c r="D46" s="7" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+    </row>
+    <row r="47" hidden="1" outlineLevel="1">
+      <c r="A47" s="5" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1">
+      <c r="A48" s="5" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+    </row>
+    <row r="49" hidden="1" outlineLevel="1">
+      <c r="A49" s="5" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1">
+      <c r="A50" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+    </row>
+    <row r="51" hidden="1" outlineLevel="1">
+      <c r="A51" s="5" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+    </row>
+    <row r="52" hidden="1" outlineLevel="1">
+      <c r="A52" s="5" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="7" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+    </row>
+    <row r="53" hidden="1" outlineLevel="1">
+      <c r="A53" s="5" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="7" t="n"/>
+      <c r="D53" s="7" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+    </row>
+    <row r="54" hidden="1" outlineLevel="1">
+      <c r="A54" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+    </row>
+    <row r="55" hidden="1" outlineLevel="1">
+      <c r="A55" s="5" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+    </row>
+    <row r="56" hidden="1" outlineLevel="1">
+      <c r="A56" s="5" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="7" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+    </row>
+    <row r="57" hidden="1" outlineLevel="1">
+      <c r="A57" s="5" t="n">
+        <v>12.75</v>
+      </c>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="7" t="n"/>
+      <c r="D57" s="7" t="n"/>
+      <c r="E57" s="6" t="n"/>
+      <c r="F57" s="6" t="n"/>
+    </row>
+    <row r="58" collapsed="1">
+      <c r="A58" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>übergang</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>strobo</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F58" s="6" t="n"/>
+    </row>
+    <row r="59" hidden="1" outlineLevel="1">
+      <c r="A59" s="5" t="n">
+        <v>13.25</v>
+      </c>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="7" t="n"/>
+      <c r="E59" s="6" t="n"/>
+      <c r="F59" s="6" t="n"/>
+    </row>
+    <row r="60" collapsed="1">
+      <c r="A60" s="5" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>chorus 1</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
           <t>action</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E60" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="F10" s="6">
-        <f>$C$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="n">
+      <c r="F60" s="6" t="n"/>
+    </row>
+    <row r="61" hidden="1" outlineLevel="1">
+      <c r="A61" s="5" t="n">
+        <v>13.75</v>
+      </c>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="7" t="n"/>
+      <c r="D61" s="7" t="n"/>
+      <c r="E61" s="6" t="n"/>
+      <c r="F61" s="6" t="n"/>
+    </row>
+    <row r="62" hidden="1" outlineLevel="1">
+      <c r="A62" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="7" t="n"/>
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="6" t="n"/>
+    </row>
+    <row r="63" hidden="1" outlineLevel="1">
+      <c r="A63" s="5" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="7" t="n"/>
+      <c r="D63" s="7" t="n"/>
+      <c r="E63" s="6" t="n"/>
+      <c r="F63" s="6" t="n"/>
+    </row>
+    <row r="64" hidden="1" outlineLevel="1">
+      <c r="A64" s="5" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="7" t="n"/>
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
+    </row>
+    <row r="65" hidden="1" outlineLevel="1">
+      <c r="A65" s="5" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="7" t="n"/>
+      <c r="D65" s="7" t="n"/>
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
+    </row>
+    <row r="66" hidden="1" outlineLevel="1">
+      <c r="A66" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="7" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="6" t="n"/>
+    </row>
+    <row r="67" hidden="1" outlineLevel="1">
+      <c r="A67" s="5" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="7" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+    </row>
+    <row r="68" hidden="1" outlineLevel="1">
+      <c r="A68" s="5" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="7" t="n"/>
+      <c r="D68" s="7" t="n"/>
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="6" t="n"/>
+    </row>
+    <row r="69" hidden="1" outlineLevel="1">
+      <c r="A69" s="5" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="7" t="n"/>
+      <c r="D69" s="7" t="n"/>
+      <c r="E69" s="6" t="n"/>
+      <c r="F69" s="6" t="n"/>
+    </row>
+    <row r="70" hidden="1" outlineLevel="1">
+      <c r="A70" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="7" t="n"/>
+      <c r="D70" s="7" t="n"/>
+      <c r="E70" s="6" t="n"/>
+      <c r="F70" s="6" t="n"/>
+    </row>
+    <row r="71" hidden="1" outlineLevel="1">
+      <c r="A71" s="5" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="7" t="n"/>
+      <c r="D71" s="7" t="n"/>
+      <c r="E71" s="6" t="n"/>
+      <c r="F71" s="6" t="n"/>
+    </row>
+    <row r="72" hidden="1" outlineLevel="1">
+      <c r="A72" s="5" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="7" t="n"/>
+      <c r="D72" s="7" t="n"/>
+      <c r="E72" s="6" t="n"/>
+      <c r="F72" s="6" t="n"/>
+    </row>
+    <row r="73" hidden="1" outlineLevel="1">
+      <c r="A73" s="5" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="B73" s="6" t="n"/>
+      <c r="C73" s="7" t="n"/>
+      <c r="D73" s="7" t="n"/>
+      <c r="E73" s="6" t="n"/>
+      <c r="F73" s="6" t="n"/>
+    </row>
+    <row r="74" hidden="1" outlineLevel="1">
+      <c r="A74" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B74" s="6" t="n"/>
+      <c r="C74" s="7" t="n"/>
+      <c r="D74" s="7" t="n"/>
+      <c r="E74" s="6" t="n"/>
+      <c r="F74" s="6" t="n"/>
+    </row>
+    <row r="75" hidden="1" outlineLevel="1">
+      <c r="A75" s="5" t="n">
+        <v>17.25</v>
+      </c>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="7" t="n"/>
+      <c r="D75" s="7" t="n"/>
+      <c r="E75" s="6" t="n"/>
+      <c r="F75" s="6" t="n"/>
+    </row>
+    <row r="76" hidden="1" outlineLevel="1">
+      <c r="A76" s="5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="7" t="n"/>
+      <c r="D76" s="7" t="n"/>
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="6" t="n"/>
+    </row>
+    <row r="77" hidden="1" outlineLevel="1">
+      <c r="A77" s="5" t="n">
+        <v>17.75</v>
+      </c>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="7" t="n"/>
+      <c r="D77" s="7" t="n"/>
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="6" t="n"/>
+    </row>
+    <row r="78" hidden="1" outlineLevel="1">
+      <c r="A78" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="7" t="n"/>
+      <c r="D78" s="7" t="n"/>
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="6" t="n"/>
+    </row>
+    <row r="79" hidden="1" outlineLevel="1">
+      <c r="A79" s="5" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="7" t="n"/>
+      <c r="D79" s="7" t="n"/>
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="6" t="n"/>
+    </row>
+    <row r="80" hidden="1" outlineLevel="1">
+      <c r="A80" s="5" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="7" t="n"/>
+      <c r="D80" s="7" t="n"/>
+      <c r="E80" s="6" t="n"/>
+      <c r="F80" s="6" t="n"/>
+    </row>
+    <row r="81" hidden="1" outlineLevel="1">
+      <c r="A81" s="5" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="7" t="n"/>
+      <c r="D81" s="7" t="n"/>
+      <c r="E81" s="6" t="n"/>
+      <c r="F81" s="6" t="n"/>
+    </row>
+    <row r="82" hidden="1" outlineLevel="1">
+      <c r="A82" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="7" t="n"/>
+      <c r="D82" s="7" t="n"/>
+      <c r="E82" s="6" t="n"/>
+      <c r="F82" s="6" t="n"/>
+    </row>
+    <row r="83" hidden="1" outlineLevel="1">
+      <c r="A83" s="5" t="n">
+        <v>19.25</v>
+      </c>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="7" t="n"/>
+      <c r="D83" s="7" t="n"/>
+      <c r="E83" s="6" t="n"/>
+      <c r="F83" s="6" t="n"/>
+    </row>
+    <row r="84" hidden="1" outlineLevel="1">
+      <c r="A84" s="5" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="7" t="n"/>
+      <c r="D84" s="7" t="n"/>
+      <c r="E84" s="6" t="n"/>
+      <c r="F84" s="6" t="n"/>
+    </row>
+    <row r="85" hidden="1" outlineLevel="1">
+      <c r="A85" s="5" t="n">
+        <v>19.75</v>
+      </c>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="7" t="n"/>
+      <c r="D85" s="7" t="n"/>
+      <c r="E85" s="6" t="n"/>
+      <c r="F85" s="6" t="n"/>
+    </row>
+    <row r="86" hidden="1" outlineLevel="1">
+      <c r="A86" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="7" t="n"/>
+      <c r="D86" s="7" t="n"/>
+      <c r="E86" s="6" t="n"/>
+      <c r="F86" s="6" t="n"/>
+    </row>
+    <row r="87" hidden="1" outlineLevel="1">
+      <c r="A87" s="5" t="n">
+        <v>20.25</v>
+      </c>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="7" t="n"/>
+      <c r="D87" s="7" t="n"/>
+      <c r="E87" s="6" t="n"/>
+      <c r="F87" s="6" t="n"/>
+    </row>
+    <row r="88" hidden="1" outlineLevel="1">
+      <c r="A88" s="5" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="7" t="n"/>
+      <c r="D88" s="7" t="n"/>
+      <c r="E88" s="6" t="n"/>
+      <c r="F88" s="6" t="n"/>
+    </row>
+    <row r="89" hidden="1" outlineLevel="1">
+      <c r="A89" s="5" t="n">
+        <v>20.75</v>
+      </c>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="7" t="n"/>
+      <c r="D89" s="7" t="n"/>
+      <c r="E89" s="6" t="n"/>
+      <c r="F89" s="6" t="n"/>
+    </row>
+    <row r="90" hidden="1" outlineLevel="1">
+      <c r="A90" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="7" t="n"/>
+      <c r="D90" s="7" t="n"/>
+      <c r="E90" s="6" t="n"/>
+      <c r="F90" s="6" t="n"/>
+    </row>
+    <row r="91" hidden="1" outlineLevel="1">
+      <c r="A91" s="5" t="n">
+        <v>21.25</v>
+      </c>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="7" t="n"/>
+      <c r="D91" s="7" t="n"/>
+      <c r="E91" s="6" t="n"/>
+      <c r="F91" s="6" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="n">
         <v>21.5</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>Ende</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>10 sek. BLACK</t>
         </is>
       </c>
-      <c r="E11" t="n">
+      <c r="E92" t="n">
         <v>0</v>
-      </c>
-      <c r="F11">
-        <f>$C$3</f>
-        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Raster-Tabelle: Gliederung in drei Ebenen (Parts, volle Takte, Viertel)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/struktur-vorlage.xlsx
+++ b/songs/struktur-vorlage.xlsx
@@ -572,11 +572,11 @@
       <c r="F6" s="6" t="n"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Zwischenzeilen (von takt ohne Songpart) = eine Zeile je Vierteltakt, eingeklappt: Plus am linken Rand öffnet einen Part, der Knopf 2 oben links alle. Leer = der Effekt des Parts läuft weiter. Ein Änderungswunsch dort gilt genau für diese Stelle. Ein Songpart-Name dort macht daraus einen neuen Part.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" hidden="1" outlineLevel="1">
+          <t>Zwischenzeilen (von takt ohne Songpart) = eine Zeile je Vierteltakt, eingeklappt in drei Ebenen (Knöpfe oben links: 1 = nur Parts, 2 = dazu volle Takte, 3 = dazu Viertel; Plus am linken Rand öffnet einen Part bzw. Takt). Leer = der Effekt des Parts läuft weiter. Ein Änderungswunsch dort gilt genau für diese Stelle. Ein Songpart-Name dort macht daraus einen neuen Part.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" hidden="1" outlineLevel="2">
       <c r="A7" s="5" t="n">
         <v>0.25</v>
       </c>
@@ -587,7 +587,7 @@
       <c r="F7" s="6" t="n"/>
       <c r="H7" s="2" t="n"/>
     </row>
-    <row r="8" hidden="1" outlineLevel="1">
+    <row r="8" hidden="1" outlineLevel="2">
       <c r="A8" s="5" t="n">
         <v>0.5</v>
       </c>
@@ -598,7 +598,7 @@
       <c r="F8" s="6" t="n"/>
       <c r="H8" s="2" t="n"/>
     </row>
-    <row r="9" hidden="1" outlineLevel="1">
+    <row r="9" hidden="1" outlineLevel="2">
       <c r="A9" s="5" t="n">
         <v>0.75</v>
       </c>
@@ -629,7 +629,7 @@
       </c>
       <c r="F10" s="6" t="n"/>
     </row>
-    <row r="11" hidden="1" outlineLevel="1">
+    <row r="11" hidden="1" outlineLevel="2">
       <c r="A11" s="5" t="n">
         <v>1.25</v>
       </c>
@@ -639,7 +639,7 @@
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
     </row>
-    <row r="12" hidden="1" outlineLevel="1">
+    <row r="12" hidden="1" outlineLevel="2">
       <c r="A12" s="5" t="n">
         <v>1.5</v>
       </c>
@@ -649,7 +649,7 @@
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
     </row>
-    <row r="13" hidden="1" outlineLevel="1">
+    <row r="13" hidden="1" outlineLevel="2">
       <c r="A13" s="5" t="n">
         <v>1.75</v>
       </c>
@@ -659,7 +659,7 @@
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
     </row>
-    <row r="14" hidden="1" outlineLevel="1">
+    <row r="14" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A14" s="5" t="n">
         <v>2</v>
       </c>
@@ -669,7 +669,7 @@
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
     </row>
-    <row r="15" hidden="1" outlineLevel="1">
+    <row r="15" hidden="1" outlineLevel="2">
       <c r="A15" s="5" t="n">
         <v>2.25</v>
       </c>
@@ -679,7 +679,7 @@
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
     </row>
-    <row r="16" hidden="1" outlineLevel="1">
+    <row r="16" hidden="1" outlineLevel="2">
       <c r="A16" s="5" t="n">
         <v>2.5</v>
       </c>
@@ -689,7 +689,7 @@
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
     </row>
-    <row r="17" hidden="1" outlineLevel="1">
+    <row r="17" hidden="1" outlineLevel="2">
       <c r="A17" s="5" t="n">
         <v>2.75</v>
       </c>
@@ -699,7 +699,7 @@
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
     </row>
-    <row r="18" hidden="1" outlineLevel="1">
+    <row r="18" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A18" s="5" t="n">
         <v>3</v>
       </c>
@@ -709,7 +709,7 @@
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
     </row>
-    <row r="19" hidden="1" outlineLevel="1">
+    <row r="19" hidden="1" outlineLevel="2">
       <c r="A19" s="5" t="n">
         <v>3.25</v>
       </c>
@@ -719,7 +719,7 @@
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
     </row>
-    <row r="20" hidden="1" outlineLevel="1">
+    <row r="20" hidden="1" outlineLevel="2">
       <c r="A20" s="5" t="n">
         <v>3.5</v>
       </c>
@@ -729,7 +729,7 @@
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
     </row>
-    <row r="21" hidden="1" outlineLevel="1">
+    <row r="21" hidden="1" outlineLevel="2">
       <c r="A21" s="5" t="n">
         <v>3.75</v>
       </c>
@@ -739,7 +739,7 @@
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
     </row>
-    <row r="22" hidden="1" outlineLevel="1">
+    <row r="22" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A22" s="5" t="n">
         <v>4</v>
       </c>
@@ -749,7 +749,7 @@
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
     </row>
-    <row r="23" hidden="1" outlineLevel="1">
+    <row r="23" hidden="1" outlineLevel="2">
       <c r="A23" s="5" t="n">
         <v>4.25</v>
       </c>
@@ -759,7 +759,7 @@
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
     </row>
-    <row r="24" hidden="1" outlineLevel="1">
+    <row r="24" hidden="1" outlineLevel="2">
       <c r="A24" s="5" t="n">
         <v>4.5</v>
       </c>
@@ -769,7 +769,7 @@
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
     </row>
-    <row r="25" hidden="1" outlineLevel="1">
+    <row r="25" hidden="1" outlineLevel="2">
       <c r="A25" s="5" t="n">
         <v>4.75</v>
       </c>
@@ -795,7 +795,7 @@
       </c>
       <c r="F26" s="6" t="n"/>
     </row>
-    <row r="27" hidden="1" outlineLevel="1">
+    <row r="27" hidden="1" outlineLevel="2">
       <c r="A27" s="5" t="n">
         <v>5.25</v>
       </c>
@@ -805,7 +805,7 @@
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
     </row>
-    <row r="28" hidden="1" outlineLevel="1">
+    <row r="28" hidden="1" outlineLevel="2">
       <c r="A28" s="5" t="n">
         <v>5.5</v>
       </c>
@@ -815,7 +815,7 @@
       <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
     </row>
-    <row r="29" hidden="1" outlineLevel="1">
+    <row r="29" hidden="1" outlineLevel="2">
       <c r="A29" s="5" t="n">
         <v>5.75</v>
       </c>
@@ -825,7 +825,7 @@
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
     </row>
-    <row r="30" hidden="1" outlineLevel="1">
+    <row r="30" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A30" s="5" t="n">
         <v>6</v>
       </c>
@@ -835,7 +835,7 @@
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
     </row>
-    <row r="31" hidden="1" outlineLevel="1">
+    <row r="31" hidden="1" outlineLevel="2">
       <c r="A31" s="5" t="n">
         <v>6.25</v>
       </c>
@@ -845,7 +845,7 @@
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
     </row>
-    <row r="32" hidden="1" outlineLevel="1">
+    <row r="32" hidden="1" outlineLevel="2">
       <c r="A32" s="5" t="n">
         <v>6.5</v>
       </c>
@@ -855,7 +855,7 @@
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
     </row>
-    <row r="33" hidden="1" outlineLevel="1">
+    <row r="33" hidden="1" outlineLevel="2">
       <c r="A33" s="5" t="n">
         <v>6.75</v>
       </c>
@@ -865,7 +865,7 @@
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
     </row>
-    <row r="34" hidden="1" outlineLevel="1">
+    <row r="34" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A34" s="5" t="n">
         <v>7</v>
       </c>
@@ -875,7 +875,7 @@
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
     </row>
-    <row r="35" hidden="1" outlineLevel="1">
+    <row r="35" hidden="1" outlineLevel="2">
       <c r="A35" s="5" t="n">
         <v>7.25</v>
       </c>
@@ -885,7 +885,7 @@
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
     </row>
-    <row r="36" hidden="1" outlineLevel="1">
+    <row r="36" hidden="1" outlineLevel="2">
       <c r="A36" s="5" t="n">
         <v>7.5</v>
       </c>
@@ -895,7 +895,7 @@
       <c r="E36" s="6" t="n"/>
       <c r="F36" s="6" t="n"/>
     </row>
-    <row r="37" hidden="1" outlineLevel="1">
+    <row r="37" hidden="1" outlineLevel="2">
       <c r="A37" s="5" t="n">
         <v>7.75</v>
       </c>
@@ -905,7 +905,7 @@
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
     </row>
-    <row r="38" hidden="1" outlineLevel="1">
+    <row r="38" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A38" s="5" t="n">
         <v>8</v>
       </c>
@@ -915,7 +915,7 @@
       <c r="E38" s="6" t="n"/>
       <c r="F38" s="6" t="n"/>
     </row>
-    <row r="39" hidden="1" outlineLevel="1">
+    <row r="39" hidden="1" outlineLevel="2">
       <c r="A39" s="5" t="n">
         <v>8.25</v>
       </c>
@@ -925,7 +925,7 @@
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
     </row>
-    <row r="40" hidden="1" outlineLevel="1">
+    <row r="40" hidden="1" outlineLevel="2">
       <c r="A40" s="5" t="n">
         <v>8.5</v>
       </c>
@@ -935,7 +935,7 @@
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="6" t="n"/>
     </row>
-    <row r="41" hidden="1" outlineLevel="1">
+    <row r="41" hidden="1" outlineLevel="2">
       <c r="A41" s="5" t="n">
         <v>8.75</v>
       </c>
@@ -945,7 +945,7 @@
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
     </row>
-    <row r="42" hidden="1" outlineLevel="1">
+    <row r="42" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A42" s="5" t="n">
         <v>9</v>
       </c>
@@ -955,7 +955,7 @@
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="6" t="n"/>
     </row>
-    <row r="43" hidden="1" outlineLevel="1">
+    <row r="43" hidden="1" outlineLevel="2">
       <c r="A43" s="5" t="n">
         <v>9.25</v>
       </c>
@@ -965,7 +965,7 @@
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
     </row>
-    <row r="44" hidden="1" outlineLevel="1">
+    <row r="44" hidden="1" outlineLevel="2">
       <c r="A44" s="5" t="n">
         <v>9.5</v>
       </c>
@@ -975,7 +975,7 @@
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="6" t="n"/>
     </row>
-    <row r="45" hidden="1" outlineLevel="1">
+    <row r="45" hidden="1" outlineLevel="2">
       <c r="A45" s="5" t="n">
         <v>9.75</v>
       </c>
@@ -985,7 +985,7 @@
       <c r="E45" s="6" t="n"/>
       <c r="F45" s="6" t="n"/>
     </row>
-    <row r="46" hidden="1" outlineLevel="1">
+    <row r="46" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A46" s="5" t="n">
         <v>10</v>
       </c>
@@ -995,7 +995,7 @@
       <c r="E46" s="6" t="n"/>
       <c r="F46" s="6" t="n"/>
     </row>
-    <row r="47" hidden="1" outlineLevel="1">
+    <row r="47" hidden="1" outlineLevel="2">
       <c r="A47" s="5" t="n">
         <v>10.25</v>
       </c>
@@ -1005,7 +1005,7 @@
       <c r="E47" s="6" t="n"/>
       <c r="F47" s="6" t="n"/>
     </row>
-    <row r="48" hidden="1" outlineLevel="1">
+    <row r="48" hidden="1" outlineLevel="2">
       <c r="A48" s="5" t="n">
         <v>10.5</v>
       </c>
@@ -1015,7 +1015,7 @@
       <c r="E48" s="6" t="n"/>
       <c r="F48" s="6" t="n"/>
     </row>
-    <row r="49" hidden="1" outlineLevel="1">
+    <row r="49" hidden="1" outlineLevel="2">
       <c r="A49" s="5" t="n">
         <v>10.75</v>
       </c>
@@ -1025,7 +1025,7 @@
       <c r="E49" s="6" t="n"/>
       <c r="F49" s="6" t="n"/>
     </row>
-    <row r="50" hidden="1" outlineLevel="1">
+    <row r="50" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A50" s="5" t="n">
         <v>11</v>
       </c>
@@ -1035,7 +1035,7 @@
       <c r="E50" s="6" t="n"/>
       <c r="F50" s="6" t="n"/>
     </row>
-    <row r="51" hidden="1" outlineLevel="1">
+    <row r="51" hidden="1" outlineLevel="2">
       <c r="A51" s="5" t="n">
         <v>11.25</v>
       </c>
@@ -1045,7 +1045,7 @@
       <c r="E51" s="6" t="n"/>
       <c r="F51" s="6" t="n"/>
     </row>
-    <row r="52" hidden="1" outlineLevel="1">
+    <row r="52" hidden="1" outlineLevel="2">
       <c r="A52" s="5" t="n">
         <v>11.5</v>
       </c>
@@ -1055,7 +1055,7 @@
       <c r="E52" s="6" t="n"/>
       <c r="F52" s="6" t="n"/>
     </row>
-    <row r="53" hidden="1" outlineLevel="1">
+    <row r="53" hidden="1" outlineLevel="2">
       <c r="A53" s="5" t="n">
         <v>11.75</v>
       </c>
@@ -1065,7 +1065,7 @@
       <c r="E53" s="6" t="n"/>
       <c r="F53" s="6" t="n"/>
     </row>
-    <row r="54" hidden="1" outlineLevel="1">
+    <row r="54" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A54" s="5" t="n">
         <v>12</v>
       </c>
@@ -1075,7 +1075,7 @@
       <c r="E54" s="6" t="n"/>
       <c r="F54" s="6" t="n"/>
     </row>
-    <row r="55" hidden="1" outlineLevel="1">
+    <row r="55" hidden="1" outlineLevel="2">
       <c r="A55" s="5" t="n">
         <v>12.25</v>
       </c>
@@ -1085,7 +1085,7 @@
       <c r="E55" s="6" t="n"/>
       <c r="F55" s="6" t="n"/>
     </row>
-    <row r="56" hidden="1" outlineLevel="1">
+    <row r="56" hidden="1" outlineLevel="2">
       <c r="A56" s="5" t="n">
         <v>12.5</v>
       </c>
@@ -1095,7 +1095,7 @@
       <c r="E56" s="6" t="n"/>
       <c r="F56" s="6" t="n"/>
     </row>
-    <row r="57" hidden="1" outlineLevel="1">
+    <row r="57" hidden="1" outlineLevel="2">
       <c r="A57" s="5" t="n">
         <v>12.75</v>
       </c>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="F58" s="6" t="n"/>
     </row>
-    <row r="59" hidden="1" outlineLevel="1">
+    <row r="59" hidden="1" outlineLevel="2">
       <c r="A59" s="5" t="n">
         <v>13.25</v>
       </c>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="F60" s="6" t="n"/>
     </row>
-    <row r="61" hidden="1" outlineLevel="1">
+    <row r="61" hidden="1" outlineLevel="2">
       <c r="A61" s="5" t="n">
         <v>13.75</v>
       </c>
@@ -1165,7 +1165,7 @@
       <c r="E61" s="6" t="n"/>
       <c r="F61" s="6" t="n"/>
     </row>
-    <row r="62" hidden="1" outlineLevel="1">
+    <row r="62" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A62" s="5" t="n">
         <v>14</v>
       </c>
@@ -1175,7 +1175,7 @@
       <c r="E62" s="6" t="n"/>
       <c r="F62" s="6" t="n"/>
     </row>
-    <row r="63" hidden="1" outlineLevel="1">
+    <row r="63" hidden="1" outlineLevel="2">
       <c r="A63" s="5" t="n">
         <v>14.25</v>
       </c>
@@ -1185,7 +1185,7 @@
       <c r="E63" s="6" t="n"/>
       <c r="F63" s="6" t="n"/>
     </row>
-    <row r="64" hidden="1" outlineLevel="1">
+    <row r="64" hidden="1" outlineLevel="2">
       <c r="A64" s="5" t="n">
         <v>14.5</v>
       </c>
@@ -1195,7 +1195,7 @@
       <c r="E64" s="6" t="n"/>
       <c r="F64" s="6" t="n"/>
     </row>
-    <row r="65" hidden="1" outlineLevel="1">
+    <row r="65" hidden="1" outlineLevel="2">
       <c r="A65" s="5" t="n">
         <v>14.75</v>
       </c>
@@ -1205,7 +1205,7 @@
       <c r="E65" s="6" t="n"/>
       <c r="F65" s="6" t="n"/>
     </row>
-    <row r="66" hidden="1" outlineLevel="1">
+    <row r="66" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A66" s="5" t="n">
         <v>15</v>
       </c>
@@ -1215,7 +1215,7 @@
       <c r="E66" s="6" t="n"/>
       <c r="F66" s="6" t="n"/>
     </row>
-    <row r="67" hidden="1" outlineLevel="1">
+    <row r="67" hidden="1" outlineLevel="2">
       <c r="A67" s="5" t="n">
         <v>15.25</v>
       </c>
@@ -1225,7 +1225,7 @@
       <c r="E67" s="6" t="n"/>
       <c r="F67" s="6" t="n"/>
     </row>
-    <row r="68" hidden="1" outlineLevel="1">
+    <row r="68" hidden="1" outlineLevel="2">
       <c r="A68" s="5" t="n">
         <v>15.5</v>
       </c>
@@ -1235,7 +1235,7 @@
       <c r="E68" s="6" t="n"/>
       <c r="F68" s="6" t="n"/>
     </row>
-    <row r="69" hidden="1" outlineLevel="1">
+    <row r="69" hidden="1" outlineLevel="2">
       <c r="A69" s="5" t="n">
         <v>15.75</v>
       </c>
@@ -1245,7 +1245,7 @@
       <c r="E69" s="6" t="n"/>
       <c r="F69" s="6" t="n"/>
     </row>
-    <row r="70" hidden="1" outlineLevel="1">
+    <row r="70" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A70" s="5" t="n">
         <v>16</v>
       </c>
@@ -1255,7 +1255,7 @@
       <c r="E70" s="6" t="n"/>
       <c r="F70" s="6" t="n"/>
     </row>
-    <row r="71" hidden="1" outlineLevel="1">
+    <row r="71" hidden="1" outlineLevel="2">
       <c r="A71" s="5" t="n">
         <v>16.25</v>
       </c>
@@ -1265,7 +1265,7 @@
       <c r="E71" s="6" t="n"/>
       <c r="F71" s="6" t="n"/>
     </row>
-    <row r="72" hidden="1" outlineLevel="1">
+    <row r="72" hidden="1" outlineLevel="2">
       <c r="A72" s="5" t="n">
         <v>16.5</v>
       </c>
@@ -1275,7 +1275,7 @@
       <c r="E72" s="6" t="n"/>
       <c r="F72" s="6" t="n"/>
     </row>
-    <row r="73" hidden="1" outlineLevel="1">
+    <row r="73" hidden="1" outlineLevel="2">
       <c r="A73" s="5" t="n">
         <v>16.75</v>
       </c>
@@ -1285,7 +1285,7 @@
       <c r="E73" s="6" t="n"/>
       <c r="F73" s="6" t="n"/>
     </row>
-    <row r="74" hidden="1" outlineLevel="1">
+    <row r="74" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A74" s="5" t="n">
         <v>17</v>
       </c>
@@ -1295,7 +1295,7 @@
       <c r="E74" s="6" t="n"/>
       <c r="F74" s="6" t="n"/>
     </row>
-    <row r="75" hidden="1" outlineLevel="1">
+    <row r="75" hidden="1" outlineLevel="2">
       <c r="A75" s="5" t="n">
         <v>17.25</v>
       </c>
@@ -1305,7 +1305,7 @@
       <c r="E75" s="6" t="n"/>
       <c r="F75" s="6" t="n"/>
     </row>
-    <row r="76" hidden="1" outlineLevel="1">
+    <row r="76" hidden="1" outlineLevel="2">
       <c r="A76" s="5" t="n">
         <v>17.5</v>
       </c>
@@ -1315,7 +1315,7 @@
       <c r="E76" s="6" t="n"/>
       <c r="F76" s="6" t="n"/>
     </row>
-    <row r="77" hidden="1" outlineLevel="1">
+    <row r="77" hidden="1" outlineLevel="2">
       <c r="A77" s="5" t="n">
         <v>17.75</v>
       </c>
@@ -1325,7 +1325,7 @@
       <c r="E77" s="6" t="n"/>
       <c r="F77" s="6" t="n"/>
     </row>
-    <row r="78" hidden="1" outlineLevel="1">
+    <row r="78" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A78" s="5" t="n">
         <v>18</v>
       </c>
@@ -1335,7 +1335,7 @@
       <c r="E78" s="6" t="n"/>
       <c r="F78" s="6" t="n"/>
     </row>
-    <row r="79" hidden="1" outlineLevel="1">
+    <row r="79" hidden="1" outlineLevel="2">
       <c r="A79" s="5" t="n">
         <v>18.25</v>
       </c>
@@ -1345,7 +1345,7 @@
       <c r="E79" s="6" t="n"/>
       <c r="F79" s="6" t="n"/>
     </row>
-    <row r="80" hidden="1" outlineLevel="1">
+    <row r="80" hidden="1" outlineLevel="2">
       <c r="A80" s="5" t="n">
         <v>18.5</v>
       </c>
@@ -1355,7 +1355,7 @@
       <c r="E80" s="6" t="n"/>
       <c r="F80" s="6" t="n"/>
     </row>
-    <row r="81" hidden="1" outlineLevel="1">
+    <row r="81" hidden="1" outlineLevel="2">
       <c r="A81" s="5" t="n">
         <v>18.75</v>
       </c>
@@ -1365,7 +1365,7 @@
       <c r="E81" s="6" t="n"/>
       <c r="F81" s="6" t="n"/>
     </row>
-    <row r="82" hidden="1" outlineLevel="1">
+    <row r="82" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A82" s="5" t="n">
         <v>19</v>
       </c>
@@ -1375,7 +1375,7 @@
       <c r="E82" s="6" t="n"/>
       <c r="F82" s="6" t="n"/>
     </row>
-    <row r="83" hidden="1" outlineLevel="1">
+    <row r="83" hidden="1" outlineLevel="2">
       <c r="A83" s="5" t="n">
         <v>19.25</v>
       </c>
@@ -1385,7 +1385,7 @@
       <c r="E83" s="6" t="n"/>
       <c r="F83" s="6" t="n"/>
     </row>
-    <row r="84" hidden="1" outlineLevel="1">
+    <row r="84" hidden="1" outlineLevel="2">
       <c r="A84" s="5" t="n">
         <v>19.5</v>
       </c>
@@ -1395,7 +1395,7 @@
       <c r="E84" s="6" t="n"/>
       <c r="F84" s="6" t="n"/>
     </row>
-    <row r="85" hidden="1" outlineLevel="1">
+    <row r="85" hidden="1" outlineLevel="2">
       <c r="A85" s="5" t="n">
         <v>19.75</v>
       </c>
@@ -1405,7 +1405,7 @@
       <c r="E85" s="6" t="n"/>
       <c r="F85" s="6" t="n"/>
     </row>
-    <row r="86" hidden="1" outlineLevel="1">
+    <row r="86" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A86" s="5" t="n">
         <v>20</v>
       </c>
@@ -1415,7 +1415,7 @@
       <c r="E86" s="6" t="n"/>
       <c r="F86" s="6" t="n"/>
     </row>
-    <row r="87" hidden="1" outlineLevel="1">
+    <row r="87" hidden="1" outlineLevel="2">
       <c r="A87" s="5" t="n">
         <v>20.25</v>
       </c>
@@ -1425,7 +1425,7 @@
       <c r="E87" s="6" t="n"/>
       <c r="F87" s="6" t="n"/>
     </row>
-    <row r="88" hidden="1" outlineLevel="1">
+    <row r="88" hidden="1" outlineLevel="2">
       <c r="A88" s="5" t="n">
         <v>20.5</v>
       </c>
@@ -1435,7 +1435,7 @@
       <c r="E88" s="6" t="n"/>
       <c r="F88" s="6" t="n"/>
     </row>
-    <row r="89" hidden="1" outlineLevel="1">
+    <row r="89" hidden="1" outlineLevel="2">
       <c r="A89" s="5" t="n">
         <v>20.75</v>
       </c>
@@ -1445,7 +1445,7 @@
       <c r="E89" s="6" t="n"/>
       <c r="F89" s="6" t="n"/>
     </row>
-    <row r="90" hidden="1" outlineLevel="1">
+    <row r="90" hidden="1" outlineLevel="1" collapsed="1">
       <c r="A90" s="5" t="n">
         <v>21</v>
       </c>
@@ -1455,7 +1455,7 @@
       <c r="E90" s="6" t="n"/>
       <c r="F90" s="6" t="n"/>
     </row>
-    <row r="91" hidden="1" outlineLevel="1">
+    <row r="91" hidden="1" outlineLevel="2">
       <c r="A91" s="5" t="n">
         <v>21.25</v>
       </c>

</xml_diff>